<commit_message>
Sunum taslağı: Yahya ÖZTÜRK eklendi (merged cell düzeltildi)
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/sunum-taslak.xlsx
+++ b/fotolar/sunum-taslak.xlsx
@@ -1726,8 +1726,16 @@
           <t>18:45 - 19:00</t>
         </is>
       </c>
-      <c r="B46" s="49" t="n"/>
-      <c r="C46" s="50" t="n"/>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Başlık</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Yahya ÖZTÜRK</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n"/>
@@ -1776,13 +1784,12 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="14">
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A46:C46"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A27:C27"/>

</xml_diff>

<commit_message>
Sunum taslağı güncel haliyle değiştirildi
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/sunum-taslak.xlsx
+++ b/fotolar/sunum-taslak.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mehme\OneDrive\Desktop\Çalıştay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{696E73AA-0EF9-4EE9-B02E-852B49757FDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F63150D9-759F-487F-BF3F-4113BA8D24E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6080" yWindow="1400" windowWidth="32710" windowHeight="18040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5640" yWindow="1910" windowWidth="32710" windowHeight="18040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="56">
   <si>
     <t>"Erzincan Jeolojik ve Kültürel Miras" Çalıştayı</t>
   </si>
@@ -106,9 +106,6 @@
   </si>
   <si>
     <t>14:30 - 14:45</t>
-  </si>
-  <si>
-    <t>KAF Zonu ve Ötelenmiş Vadiler</t>
   </si>
   <si>
     <t>Mehmet Akif TAŞ</t>
@@ -859,11 +856,9 @@
     <xf numFmtId="0" fontId="5" fillId="14" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -898,14 +893,16 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1253,18 +1250,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
     </row>
     <row r="2" spans="1:3" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
     </row>
     <row r="3" spans="1:3" ht="8" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
@@ -1272,18 +1269,18 @@
       <c r="C3" s="1"/>
     </row>
     <row r="4" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
+      <c r="B4" s="34"/>
+      <c r="C4" s="34"/>
     </row>
     <row r="5" spans="1:3" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="38" t="s">
+      <c r="A5" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="36"/>
-      <c r="C5" s="36"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
     </row>
     <row r="6" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
@@ -1319,11 +1316,11 @@
       </c>
     </row>
     <row r="9" spans="1:3" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="40" t="s">
+      <c r="A9" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="41"/>
-      <c r="C9" s="42"/>
+      <c r="B9" s="39"/>
+      <c r="C9" s="40"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
@@ -1359,11 +1356,11 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="34"/>
-      <c r="C13" s="34"/>
+      <c r="B13" s="32"/>
+      <c r="C13" s="32"/>
     </row>
     <row r="14" spans="1:3" ht="8" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
@@ -1371,18 +1368,18 @@
       <c r="C14" s="1"/>
     </row>
     <row r="15" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="48" t="s">
+      <c r="A15" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="36"/>
-      <c r="C15" s="36"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="34"/>
     </row>
     <row r="16" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="47" t="s">
+      <c r="A16" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="36"/>
-      <c r="C16" s="36"/>
+      <c r="B16" s="34"/>
+      <c r="C16" s="34"/>
     </row>
     <row r="17" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="19" t="s">
@@ -1432,41 +1429,39 @@
       <c r="A21" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B21" s="15" t="s">
+      <c r="B21" s="15"/>
+      <c r="C21" s="10" t="s">
         <v>28</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="7" t="s">
         <v>30</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B23" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23" s="10" t="s">
+    </row>
+    <row r="24" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="45" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="30" t="s">
-        <v>34</v>
-      </c>
-      <c r="B24" s="31"/>
-      <c r="C24" s="32"/>
+      <c r="B24" s="46"/>
+      <c r="C24" s="47"/>
     </row>
     <row r="25" spans="1:3" ht="8" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1"/>
@@ -1474,18 +1469,18 @@
       <c r="C25" s="1"/>
     </row>
     <row r="26" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="46" t="s">
-        <v>35</v>
-      </c>
-      <c r="B26" s="36"/>
-      <c r="C26" s="36"/>
+      <c r="A26" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" s="34"/>
+      <c r="C26" s="34"/>
     </row>
     <row r="27" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="B27" s="36"/>
-      <c r="C27" s="36"/>
+      <c r="B27" s="34"/>
+      <c r="C27" s="34"/>
     </row>
     <row r="28" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
@@ -1500,40 +1495,40 @@
     </row>
     <row r="29" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C29" s="7" t="s">
         <v>36</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B30" s="9" t="s">
         <v>8</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>8</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="50" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B32" s="51"/>
       <c r="C32" s="52"/>
@@ -1544,18 +1539,18 @@
       <c r="C33" s="1"/>
     </row>
     <row r="34" spans="1:3" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="B34" s="36"/>
-      <c r="C34" s="36"/>
+      <c r="A34" s="42" t="s">
+        <v>40</v>
+      </c>
+      <c r="B34" s="34"/>
+      <c r="C34" s="34"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A35" s="35" t="s">
+      <c r="A35" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="B35" s="36"/>
-      <c r="C35" s="36"/>
+      <c r="B35" s="34"/>
+      <c r="C35" s="34"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
@@ -1570,68 +1565,68 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C37" s="7" t="s">
         <v>42</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C38" s="10" t="s">
         <v>44</v>
-      </c>
-      <c r="B38" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C38" s="10" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C39" s="7" t="s">
         <v>46</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" s="16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B40" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="C40" s="18" t="s">
         <v>49</v>
-      </c>
-      <c r="C40" s="18" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B41" s="12" t="s">
         <v>8</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B42" s="21" t="s">
         <v>8</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
@@ -1639,7 +1634,7 @@
       <c r="B43" s="1"/>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="C44" s="49"/>
+      <c r="C44" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>

<commit_message>
Kurul/davetli/oturum revizyonu: Düzenleme +3, Davetli -4, oturumlar 5/4/3/6
- Düzenleme Kurulu: +Melike Bekar, +Ayşegül Kesik (Rukiye Öz altına), +Samet Altınbilek (Fatih Orhan altına) — static + 3 dil.

- Davetli Konuşmacılar'dan kaldırıldı: İbrahim Kopar, Samet Altınbilek, Gülpınar Akbulut (üçü Bilim Kurulu'nda kaldı); Fethi Ahmet Yüksel her yerden silindi (kart+oturum+PDF).

- Oturumlar 5/6/4/7 -> 5/4/3/6: Çağlayan -Kopar -Altınbilek; Kemaliye -Yüksel; Karma -Akbulut +Seven·Öztürk. M.A.Taş 'Polat Gölü' başlığı; Seven · Yahya Öztürk (Tonbul gösterimden çıkarıldı).

- İndirilebilir kurullar/program-taslak/sunum-taslak xlsx güncellendi.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/sunum-taslak.xlsx
+++ b/fotolar/sunum-taslak.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="5640" yWindow="1910" windowWidth="32710" windowHeight="18040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -215,7 +215,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -224,10 +224,51 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D0D0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="FFD0D0D0"/>
+        <color rgb="FF999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
       </top>
       <bottom style="thin">
         <color rgb="FFD0D0D0"/>
@@ -236,13 +277,13 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFD0D0D0"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD0D0D0"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD0D0D0"/>
+        <color rgb="FF999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
       </top>
       <bottom style="thin">
         <color rgb="FFD0D0D0"/>
@@ -251,148 +292,59 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFD0D0D0"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD0D0D0"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD0D0D0"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
+        <color rgb="FF999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
       <right/>
       <top style="thin">
-        <color rgb="FF999999"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD0D0D0"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD0D0D0"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF999999"/>
+        <color rgb="FFD0D0D0"/>
       </top>
       <bottom style="thin">
         <color rgb="FFD0D0D0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF999999"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD0D0D0"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF999999"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD0D0D0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF999999"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD0D0D0"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD0D0D0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD0D0D0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD0D0D0"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF999999"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF999999"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD0D0D0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD0D0D0"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF999999"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD0D0D0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD0D0D0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF999999"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FFD0D0D0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD0D0D0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF999999"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD0D0D0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD0D0D0"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFD0D0D0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF999999"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF999999"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD0D0D0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF999999"/>
       </bottom>
       <diagonal/>
     </border>
@@ -563,26 +515,6 @@
       <bottom style="thin">
         <color rgb="FF999999"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFD0D0D0"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF999999"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD0D0D0"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -602,106 +534,104 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="14" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -711,11 +641,9 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -728,11 +656,9 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -740,15 +666,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1118,50 +1035,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col width="20.90625" customWidth="1" style="34" min="1" max="1"/>
-    <col width="50.90625" customWidth="1" style="34" min="2" max="2"/>
-    <col width="40.81640625" customWidth="1" style="34" min="3" max="3"/>
-    <col width="10.81640625" customWidth="1" style="34" min="10" max="10"/>
-    <col width="48.36328125" customWidth="1" style="34" min="11" max="11"/>
+    <col width="56.453125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="104" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="40.81640625" customWidth="1" min="3" max="3"/>
+    <col width="10.81640625" customWidth="1" min="10" max="10"/>
+    <col width="48.36328125" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" s="34">
-      <c r="A1" s="35" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="33" t="inlineStr">
         <is>
           <t>"Erzincan Jeolojik ve Kültürel Miras" Çalıştayı</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="25" customHeight="1" s="34">
-      <c r="A2" s="37" t="inlineStr">
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="35" t="inlineStr">
         <is>
           <t>📅  18 Haziran (Perşembe) 2026</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="8" customHeight="1" s="34">
+    <row r="3" ht="8" customHeight="1">
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="1" t="n"/>
       <c r="C3" s="1" t="n"/>
     </row>
-    <row r="4" ht="15.5" customHeight="1" s="34">
-      <c r="A4" s="43" t="inlineStr">
+    <row r="4" ht="15.5" customHeight="1">
+      <c r="A4" s="39" t="inlineStr">
         <is>
           <t>OTURUM 1 — ERZİNCAN-OTLUKBELİ OTURUMU</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="24.5" customHeight="1" s="34">
-      <c r="A5" s="36" t="inlineStr">
+    <row r="5" ht="24.5" customHeight="1">
+      <c r="A5" s="34" t="inlineStr">
         <is>
           <t>Oturum Yürütücüleri:</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15.5" customHeight="1" s="34">
+    <row r="6" ht="15.5" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>SAAT</t>
@@ -1212,8 +1129,8 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="20.5" customHeight="1" s="34">
-      <c r="A9" s="38" t="inlineStr">
+    <row r="9" ht="20.5" customHeight="1">
+      <c r="A9" s="36" t="inlineStr">
         <is>
           <t>10:30 - 10:45  ☕ Çay / Kahve Arası</t>
         </is>
@@ -1277,26 +1194,26 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="8" customHeight="1" s="34">
+    <row r="14" ht="8" customHeight="1">
       <c r="A14" s="1" t="n"/>
       <c r="B14" s="1" t="n"/>
       <c r="C14" s="1" t="n"/>
     </row>
-    <row r="15" ht="21" customHeight="1" s="34">
-      <c r="A15" s="49" t="inlineStr">
+    <row r="15" ht="21" customHeight="1">
+      <c r="A15" s="43" t="inlineStr">
         <is>
           <t>OTURUM 2 — ERZİNCAN-ÇAĞLAYAN OTURUMU</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="21" customHeight="1" s="34">
-      <c r="A16" s="48" t="inlineStr">
+    <row r="16" ht="21" customHeight="1">
+      <c r="A16" s="42" t="inlineStr">
         <is>
           <t>Oturum Yürütücüleri:</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="19" customHeight="1" s="34">
+    <row r="17" ht="19" customHeight="1">
       <c r="A17" s="19" t="inlineStr">
         <is>
           <t>SAAT</t>
@@ -1313,7 +1230,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="19" customHeight="1" s="34">
+    <row r="18" ht="19" customHeight="1">
       <c r="A18" s="23" t="inlineStr">
         <is>
           <t>13:30 - 14:00</t>
@@ -1330,7 +1247,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="19" customHeight="1" s="34">
+    <row r="19" ht="19" customHeight="1">
       <c r="A19" s="25" t="inlineStr">
         <is>
           <t>14:00 - 14:15</t>
@@ -1343,7 +1260,7 @@
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>MTA Ekibi-1 (Ali ERGEN)</t>
+          <t>Ali ERGEN</t>
         </is>
       </c>
     </row>
@@ -1355,12 +1272,12 @@
       </c>
       <c r="B20" s="27" t="inlineStr">
         <is>
-          <t>Başlık</t>
+          <t>Polat Gölü'nün Jeolojik-Jeomorfolojik Önemi ve Jeomiras Potansiyeli</t>
         </is>
       </c>
       <c r="C20" s="29" t="inlineStr">
         <is>
-          <t>İbrahim KOPAR</t>
+          <t>Mehmet Akif TAŞ</t>
         </is>
       </c>
     </row>
@@ -1370,292 +1287,262 @@
           <t>14:30 - 14:45</t>
         </is>
       </c>
-      <c r="B21" s="15" t="n"/>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>Başlık</t>
+        </is>
+      </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Mehmet Akif TAŞ</t>
+          <t>Volkan DEDE / Kuddusi ZORLU</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>14:45 - 15:00</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>15:15 - 15:30  ☕ Çay / Kahve Arası</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n"/>
+      <c r="B23" s="1" t="n"/>
+      <c r="C23" s="1" t="n"/>
+    </row>
+    <row r="24" ht="19" customHeight="1">
+      <c r="A24" s="40" t="inlineStr">
+        <is>
+          <t>OTURUM 3 — ERZİNCAN-KEMALİYE OTURUMU</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="8" customHeight="1">
+      <c r="A25" s="37" t="inlineStr">
+        <is>
+          <t>Oturum Yürütücüleri:</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>SAAT</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>BİLDİRİ BAŞLIĞI</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>SUNUM YAPAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>15:30 - 15:45</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Başlık</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>Samet ALTINBİLEK</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>15:00 - 15:15</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Kenan İNAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>15:45 - 16:00</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>Başlık</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>Volkan DEDE / Kuddusi ZORLU</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="19" customHeight="1" s="34">
-      <c r="A24" s="45" t="inlineStr">
-        <is>
-          <t>15:15 - 15:30  ☕ Çay / Kahve Arası</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="8" customHeight="1" s="34">
-      <c r="A25" s="1" t="n"/>
-      <c r="B25" s="1" t="n"/>
-      <c r="C25" s="1" t="n"/>
-    </row>
-    <row r="26" ht="18" customHeight="1" s="34">
-      <c r="A26" s="44" t="inlineStr">
-        <is>
-          <t>OTURUM 3 — ERZİNCAN-KEMALİYE OTURUMU</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="18" customHeight="1" s="34">
-      <c r="A27" s="41" t="inlineStr">
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Erdal AKPINAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>16:00 - 16:15</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Başlık</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Vedat Güngör/Mustafa BAYAM (Erzincan Müze Müd.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="17.5" customHeight="1">
+      <c r="A30" s="44" t="inlineStr">
+        <is>
+          <t>16:15 - 16:30  ☕ Çay / Kahve Arası</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n"/>
+      <c r="B31" s="1" t="n"/>
+      <c r="C31" s="1" t="n"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="38" t="inlineStr">
+        <is>
+          <t>OTURUM 4 — ERZİNCAN KARMA OTURUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="8" customHeight="1">
+      <c r="A33" s="32" t="inlineStr">
         <is>
           <t>Oturum Yürütücüleri:</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="18" customHeight="1" s="34">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="34" ht="15.5" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>SAAT</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>BİLDİRİ BAŞLIĞI</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>SUNUM YAPAN</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1" s="34">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>15:30 - 15:45</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>16:45 - 17:00</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>Başlık</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>Kenan İNAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="17.5" customHeight="1" s="34">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>15:45 - 16:00</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>Başlık</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>Erdal AKPINAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>16:00 - 16:15</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>Başlık</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>Vedat Güngör/Mustafa BAYAM (Erzincan Müze Müd.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1" s="34">
-      <c r="A32" s="53" t="inlineStr">
-        <is>
-          <t>16:15 - 16:30  ☕ Çay / Kahve Arası</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="8" customHeight="1" s="34">
-      <c r="A33" s="1" t="n"/>
-      <c r="B33" s="1" t="n"/>
-      <c r="C33" s="1" t="n"/>
-    </row>
-    <row r="34" ht="15.5" customHeight="1" s="34">
-      <c r="A34" s="42" t="inlineStr">
-        <is>
-          <t>OTURUM 4 — ERZİNCAN KARMA OTURUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="33" t="inlineStr">
-        <is>
-          <t>Oturum Yürütücüleri:</t>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Ali DEMİRSOY</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>SAAT</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>BİLDİRİ BAŞLIĞI</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>SUNUM YAPAN</t>
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>17:00 - 17:15</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Kemaliye'nin Jeolojisi, Doğa Değerleri, Antropojenik Tehlikeler ve Koruma Statüsü</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>Eşref ATABEY</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>16:45 - 17:00</t>
+          <t>17:15 - 17:30</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
+          <t>Kuzey Anadolu Fayı'nın Magmatik İzlerinden Jeolojik Mirasa: Erzincan Volkan Konilerinin Jeokimyasal ve Petrojenetik Değerlendirmesi</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Fatma TÜKEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t>17:30 - 17:45</t>
+        </is>
+      </c>
+      <c r="B38" s="17" t="inlineStr">
+        <is>
           <t>Başlık</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>Ali DEMİRSOY</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>17:00 - 17:15</t>
-        </is>
-      </c>
-      <c r="B38" s="9" t="inlineStr">
-        <is>
-          <t>Kemaliye'nin Jeolojisi, Doğa Değerleri, Antropojenik Tehlikeler ve Koruma Statüsü</t>
-        </is>
-      </c>
-      <c r="C38" s="10" t="inlineStr">
-        <is>
-          <t>Eşref ATABEY</t>
+      <c r="C38" s="18" t="inlineStr">
+        <is>
+          <t>M. Feridun ÇELİKMEN (KEMAV Başkanı)</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>17:15 - 17:30</t>
-        </is>
-      </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>17:45 - 18:00</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
         <is>
           <t>Başlık</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>Gülpınar AKBULUT</t>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>Pınar POLAT</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="16" t="inlineStr">
-        <is>
-          <t>17:30 - 17:45</t>
-        </is>
-      </c>
-      <c r="B40" s="17" t="inlineStr">
-        <is>
-          <t>Kuzey Anadolu Fayı'nın Magmatik İzlerinden Jeolojik Mirasa: Erzincan Volkan Konilerinin Jeokimyasal ve Petrojenetik Değerlendirmesi</t>
-        </is>
-      </c>
-      <c r="C40" s="18" t="inlineStr">
-        <is>
-          <t>Fatma TÜKEL</t>
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>18:00 - 18:15</t>
+        </is>
+      </c>
+      <c r="B40" s="21" t="inlineStr">
+        <is>
+          <t>Esence (Keşiş) Dağları'nda Buzul Jeomorfolojisinin Jeomiras Potansiyeli</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Mutlu SEVEN / Yahya ÖZTÜRK</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="inlineStr">
-        <is>
-          <t>17:45 - 18:00</t>
-        </is>
-      </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>Başlık</t>
-        </is>
-      </c>
-      <c r="C41" s="13" t="inlineStr">
-        <is>
-          <t>M. Feridun ÇELİKMEN (KEMAV Başkanı)</t>
-        </is>
-      </c>
+      <c r="A41" s="1" t="n"/>
+      <c r="B41" s="1" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="14" t="inlineStr">
-        <is>
-          <t>18:00 - 18:15</t>
-        </is>
-      </c>
-      <c r="B42" s="21" t="inlineStr">
-        <is>
-          <t>Başlık</t>
-        </is>
-      </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>Pınar POLAT</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="1" t="n"/>
-      <c r="B43" s="1" t="n"/>
-    </row>
-    <row r="44">
-      <c r="C44" s="30" t="n"/>
+      <c r="C42" s="30" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Davetli konuşmacılar masonry düzeni + doğrulama temizlikleri
- Konuşmacı kartları CSS sütun akışına (masonry) geçti: columns:320px,
  break-inside:avoid — kısa kartların dev boşluklu gerilmesi sona erdi
- Doğrulama denetçilerinin bulguları: yetim sp_role_dede anahtarı 3 dilden
  silindi (308 anahtar/dil); mükerrer venue_map_* satırları (TR/EN) kaldırıldı
- sunum-taslak.xlsx: C20 TAGLİASACCHİ→TAGLIASACCHI (düz I kararı);
  Yıldırım Güngör başlığı eklendi (sitede vardı, xlsx'te eksikti)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/sunum-taslak.xlsx
+++ b/fotolar/sunum-taslak.xlsx
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Başlık</t>
+          <t>Jeolojik Miras Envanter Çalışması Aşamaları</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="C20" s="29" t="inlineStr">
         <is>
-          <t>Mehmet Akif TAŞ / Pınar POLAT / Yakup ÇELİK / Ezher TAGLİASACCHİ</t>
+          <t>Mehmet Akif TAŞ / Pınar POLAT / Yakup ÇELİK / Ezher TAGLIASACCHI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Karma Oturum -> Üzümlü Oturum (Oturum 4) + sunum xlsx senkron
- Site Oturum 4 adı 'Karma' -> 'Üzümlü' (3 dil: TR 'Erzincan Üzümlü Oturum',
  EN 'Erzincan Üzümlü Session', IT 'Sessione Üzümlü Erzincan' — topic kartı,
  timeline, t4_title, d1_s10_title; statik + i18n)
- Kullanıcının güncellediği program/sunum taslakları yüklendi (Üzümlü adı)
- sunum-taslak.xlsx: CAPEZZUOLI düz-I geri-düzeltildi (kullanıcı dosyasında
  kazara Türkçe İ'ye dönmüştü; önceki karar korundu)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/sunum-taslak.xlsx
+++ b/fotolar/sunum-taslak.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1140" yWindow="1140" windowWidth="32710" windowHeight="18040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -1416,7 +1416,7 @@
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="29" t="inlineStr">
         <is>
-          <t>OTURUM 4 — ERZİNCAN KARMA OTURUM</t>
+          <t>OTURUM 4 — ERZİNCAN ÜZÜMLÜ OTURUM</t>
         </is>
       </c>
       <c r="C32" s="38" t="n"/>

</xml_diff>